<commit_message>
Committing all the files
</commit_message>
<xml_diff>
--- a/Student Credential.xlsx
+++ b/Student Credential.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="18350" windowHeight="6800"/>
+    <workbookView windowWidth="18350" windowHeight="6200"/>
   </bookViews>
   <sheets>
     <sheet name="Student Credential" sheetId="1" r:id="rId1"/>
@@ -74,7 +74,7 @@
     <t>Kashif9876@</t>
   </si>
   <si>
-    <t>Kashif</t>
+    <t>Kashif Bro</t>
   </si>
   <si>
     <t>Kashif1221@gmail.com</t>
@@ -702,7 +702,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -710,9 +710,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6" applyAlignment="1">
@@ -1265,13 +1262,13 @@
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:5">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
@@ -1291,10 +1288,10 @@
       <c r="C2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="5">
+      <c r="E2" s="4">
         <v>46037</v>
       </c>
     </row>
@@ -1308,10 +1305,10 @@
       <c r="C3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="5">
+      <c r="E3" s="4">
         <v>46050</v>
       </c>
     </row>
@@ -1325,10 +1322,10 @@
       <c r="C4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="4">
         <v>46091</v>
       </c>
     </row>

</xml_diff>